<commit_message>
Reset Philips templates to blank after importing their filled-in real data
The Blitz Call Diary and Weekly Feedback templates had real rows filled
in locally; that data (1 completed diary visit + 2 feedback survey
responses with resolvable store codes) is now imported into PH-201's
visit history via admin-visits-import. Reset both files back to blank
so the site keeps serving empty templates for future downloads.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/reports/philips/blitz-call-diary-template.xlsx
+++ b/public/reports/philips/blitz-call-diary-template.xlsx
@@ -2,15 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="7300" yWindow="600" windowWidth="21500" windowHeight="16480" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Blitz Call Diary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -26,8 +25,11 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">
@@ -39,7 +41,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000B1B3A"/>
+        <fgColor rgb="FF0B1B3A"/>
       </patternFill>
     </fill>
   </fills>
@@ -60,7 +62,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -423,14 +425,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="3" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="32" customWidth="1" min="7" max="7"/>
   </cols>
@@ -469,105 +469,6 @@
       <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Lindani Khanyile</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Checkers Boksburg</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2026-05-04</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>09:05</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Lindani Khanyile</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Dischem Alliens Nek</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>2026-05-04</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>11:00</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Missed</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Store closed for stocktake</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Mmuluki  Makhurane</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Kloppers Castle Gate</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>2026-05-05</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>10:00</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Rescheduled</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Moved to 2026-05-06</t>
         </is>
       </c>
     </row>

</xml_diff>